<commit_message>
Adding my personal info
</commit_message>
<xml_diff>
--- a/submission/Group Formation/STA380GroupForm.xlsx
+++ b/submission/Group Formation/STA380GroupForm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\49482\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/380_group_project/sta380-group-project/submission/Group Formation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8977763-ABF1-4590-AE9A-9E77F55C3BB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA01D63A-519B-A44D-B780-A27EEE3DB1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2172" yWindow="2172" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1400" yWindow="2160" windowWidth="23860" windowHeight="13320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -98,13 +98,24 @@
   </si>
   <si>
     <t>https://github.com/clara0510huang/sta380-group-project.git</t>
+  </si>
+  <si>
+    <t>Dongshuo Yang</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>yangdo35</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://github.com/yangdo35</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -115,6 +126,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -123,6 +135,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -130,6 +143,21 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -159,12 +187,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -384,17 +413,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" customWidth="1"/>
-    <col min="3" max="3" width="15.21875" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" customWidth="1"/>
     <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.21875" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -402,12 +431,12 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -415,67 +444,67 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -493,7 +522,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>13</v>
       </c>
@@ -513,47 +542,63 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22">
+        <v>1007867202</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update STA380 group formation Excel with my information
</commit_message>
<xml_diff>
--- a/submission/Group Formation/STA380GroupForm.xlsx
+++ b/submission/Group Formation/STA380GroupForm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\49482\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 winter\sta380\380project\sta380-group-project\submission\Group Formation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE00BA61-193D-4176-9DDA-C09130CEF63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16E2990-F560-40CE-AC01-EE1E41EEEA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1215" yWindow="3960" windowWidth="28800" windowHeight="15330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -115,6 +115,24 @@
   </si>
   <si>
     <t>Exponential + Normal</t>
+  </si>
+  <si>
+    <t>Qi Wang</t>
+  </si>
+  <si>
+    <t>wangq388</t>
+  </si>
+  <si>
+    <t>https://github.com/mdfkgtm</t>
+  </si>
+  <si>
+    <t>mdfkgtm</t>
+  </si>
+  <si>
+    <t>Bootstrap Estimate</t>
+  </si>
+  <si>
+    <t>Linear regression + Mean variance</t>
   </si>
 </sst>
 </file>
@@ -193,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -213,9 +231,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -432,14 +451,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.77734375" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1">
@@ -488,10 +507,16 @@
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" customHeight="1">
@@ -603,11 +628,21 @@
       <c r="A23" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="B23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1010643715</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6"/>

</xml_diff>

<commit_message>
detail changes for t2
</commit_message>
<xml_diff>
--- a/submission/Group Formation/STA380GroupForm.xlsx
+++ b/submission/Group Formation/STA380GroupForm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/380_group_project/sta380-group-project/submission/Group Formation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB631556-2DD4-6145-9A90-EDA081907AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A15E2A6-4229-C34F-A41D-2A916297FD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3560" yWindow="2440" windowWidth="28400" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1840" yWindow="2440" windowWidth="28400" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -175,9 +175,6 @@
     <t>Exponential + Gamma</t>
   </si>
   <si>
-    <t>This project uses the Boston Housing Dataset to study the bootstrap estimation of linear regression coefficients (β₀, β₁),</t>
-  </si>
-  <si>
     <t xml:space="preserve">We will use inverse-transformation method to simulate exponential and gamma distribution, including the </t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -186,11 +183,15 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">we will use the OLS estimates derived from the full dataset as our reference of true values. Then assess the bias and </t>
+    <t>This project uses the Boston Housing Dataset to study the bootstrap estimation of linear regression coefficients including</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>standard error of bootstrap estimates relatie to the "true values".</t>
+    <t xml:space="preserve">intercept and slope, we will use the OLS estimates derived from the full dataset as our reference of true values. </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Then assess the bias and standard error of bootstrap estimates relatie to the "true values".</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -414,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -499,11 +500,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1838,42 +1840,42 @@
       <c r="A12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="47" t="s">
-        <v>46</v>
+      <c r="B12" s="36" t="s">
+        <v>48</v>
       </c>
       <c r="C12" s="47"/>
       <c r="D12" s="47"/>
       <c r="E12" s="47"/>
       <c r="F12" s="47"/>
-      <c r="G12" s="46"/>
+      <c r="G12" s="48"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
     </row>
     <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="16"/>
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="44" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
+      <c r="C13" s="44"/>
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
       <c r="F13" s="44"/>
-      <c r="G13" s="6"/>
+      <c r="G13" s="49"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
     <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="16"/>
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="44" t="s">
         <v>50</v>
       </c>
       <c r="C14" s="45"/>
       <c r="D14" s="45"/>
       <c r="E14" s="45"/>
       <c r="F14" s="45"/>
-      <c r="G14" s="44"/>
+      <c r="G14" s="46"/>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
@@ -1927,7 +1929,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="39"/>
       <c r="D18" s="39"/>
@@ -1941,7 +1943,7 @@
     <row r="19" spans="1:10" ht="13.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="16"/>
       <c r="B19" s="41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="42"/>
       <c r="D19" s="42"/>
@@ -2228,7 +2230,7 @@
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B13:G13"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>

</xml_diff>